<commit_message>
Add favorites page and semicolon import lists
</commit_message>
<xml_diff>
--- a/templates/sobag-products-template.xlsx
+++ b/templates/sobag-products-template.xlsx
@@ -116,17 +116,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Подушка, Наволочка</t>
+          <t>Подушка; Наволочка</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>30x30, 35x35, 40x40, 45x45, 50x50</t>
+          <t>30x30; 35x35; 40x40; 45x45; 50x50</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Велюр, Габардин</t>
+          <t>Велюр; Габардин</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -136,7 +136,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Аниме, Животные</t>
+          <t>Аниме; Животные</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -146,7 +146,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>аниме, коты, подарок</t>
+          <t>аниме; коты; подарок</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">

</xml_diff>

<commit_message>
Support multi-category imports and duplicate guards
</commit_message>
<xml_diff>
--- a/templates/sobag-products-template.xlsx
+++ b/templates/sobag-products-template.xlsx
@@ -24,7 +24,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Категория</t>
+          <t>Категории</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -111,7 +111,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Подушки</t>
+          <t>Подушки; Наволочки</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">

</xml_diff>

<commit_message>
Add product publication statuses
</commit_message>
<xml_diff>
--- a/templates/sobag-products-template.xlsx
+++ b/templates/sobag-products-template.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:R2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -74,25 +74,30 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Статус</t>
+          <t>Статус публикации</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>Статус наличия</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>Популярность</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Папка фото</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Главное фото</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Фото галереи</t>
         </is>
@@ -161,25 +166,30 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t>draft</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>made</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>10345</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>